<commit_message>
Updated N fertiliser data
Adds N-content to Peas.
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85629D09-B1AB-4161-A7B7-4BCA3CFCA6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916EBC08-63FA-4880-A697-77B5FD265A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -2689,7 +2689,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2831,13 +2831,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Hyperlink" xfId="11" xr:uid="{27B946F3-5790-4F7E-8391-6BBF48B2CC3B}"/>
@@ -3350,7 +3346,7 @@
   <cols>
     <col min="2" max="2" width="32.90625" customWidth="1"/>
     <col min="3" max="3" width="15.36328125" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" style="63" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" customWidth="1"/>
     <col min="5" max="175" width="5.6328125" customWidth="1"/>
     <col min="176" max="176" width="5.6328125" style="1" customWidth="1"/>
     <col min="177" max="202" width="5.6328125" customWidth="1"/>
@@ -3972,7 +3968,7 @@
       <c r="C5" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="64" t="s">
+      <c r="D5" s="26" t="s">
         <v>236</v>
       </c>
       <c r="E5" s="26" t="s">
@@ -4580,7 +4576,7 @@
       <c r="C6" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="65">
+      <c r="D6" s="36">
         <f>0.9753*GL6+0.02473*AP6</f>
         <v>246.37218999999999</v>
       </c>
@@ -4629,7 +4625,7 @@
       <c r="C8" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D8" s="63" t="s">
+      <c r="D8" t="s">
         <v>401</v>
       </c>
       <c r="BC8">
@@ -4649,7 +4645,7 @@
       <c r="C9" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" t="s">
         <v>641</v>
       </c>
       <c r="FT9" s="56"/>
@@ -4664,7 +4660,7 @@
       <c r="C10" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="63" t="s">
+      <c r="D10" t="s">
         <v>635</v>
       </c>
       <c r="BC10">
@@ -4682,7 +4678,7 @@
       <c r="C11" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="63" t="s">
+      <c r="D11" t="s">
         <v>401</v>
       </c>
       <c r="BC11">
@@ -4722,7 +4718,7 @@
       <c r="C13" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="65">
+      <c r="D13" s="36">
         <f>0.7067*CI13+0.1908*BG13+0.05134*AU13+0.05098*AQ13</f>
         <v>147.54371239</v>
       </c>
@@ -4752,7 +4748,7 @@
       <c r="C14" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D14" s="63" t="s">
+      <c r="D14" t="s">
         <v>401</v>
       </c>
       <c r="BC14">
@@ -4772,7 +4768,7 @@
       <c r="C15" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" t="s">
         <v>401</v>
       </c>
       <c r="BC15">
@@ -4792,7 +4788,7 @@
       <c r="C16" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="63" t="s">
+      <c r="D16" t="s">
         <v>401</v>
       </c>
       <c r="AB16" s="19"/>
@@ -4813,7 +4809,7 @@
       <c r="C17" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="D17" t="s">
         <v>401</v>
       </c>
       <c r="BC17">
@@ -4833,7 +4829,7 @@
       <c r="C18" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" t="s">
         <v>636</v>
       </c>
       <c r="BC18">
@@ -4851,7 +4847,7 @@
       <c r="C19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="D19" t="s">
         <v>627</v>
       </c>
       <c r="FT19" s="56"/>
@@ -4866,7 +4862,7 @@
       <c r="C20" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D20" s="63" t="s">
+      <c r="D20" t="s">
         <v>401</v>
       </c>
       <c r="BC20">
@@ -4904,7 +4900,7 @@
       <c r="C22" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D22" s="63" t="s">
+      <c r="D22" t="s">
         <v>401</v>
       </c>
       <c r="BC22">
@@ -4924,7 +4920,7 @@
       <c r="C23" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" t="s">
         <v>645</v>
       </c>
     </row>
@@ -4938,7 +4934,7 @@
       <c r="C24" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="D24" t="s">
         <v>401</v>
       </c>
       <c r="BC24">
@@ -4958,7 +4954,7 @@
       <c r="C25" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" t="s">
         <v>397</v>
       </c>
       <c r="FP25">
@@ -4975,7 +4971,7 @@
       <c r="C26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="D26" t="s">
         <v>401</v>
       </c>
       <c r="BC26">
@@ -4995,7 +4991,7 @@
       <c r="C27" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" t="s">
         <v>312</v>
       </c>
       <c r="CI27">
@@ -5051,7 +5047,7 @@
       <c r="C30" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D30" s="63" t="s">
+      <c r="D30" t="s">
         <v>636</v>
       </c>
       <c r="M30" s="28"/>
@@ -5067,7 +5063,7 @@
       <c r="C31" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D31" s="63" t="s">
+      <c r="D31" t="s">
         <v>627</v>
       </c>
       <c r="FT31" s="57"/>
@@ -5097,7 +5093,7 @@
       <c r="C33" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D33" s="63" t="s">
+      <c r="D33" t="s">
         <v>397</v>
       </c>
       <c r="FP33">
@@ -5115,7 +5111,7 @@
       <c r="C34" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D34" s="65">
+      <c r="D34" s="36">
         <f>0.478*AZ34+0.269*CJ34+0.253*BX34</f>
         <v>32.094000000000001</v>
       </c>
@@ -5140,7 +5136,7 @@
       <c r="C35" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D35" s="65">
+      <c r="D35" s="36">
         <f>0.4136*CJ35+0.3486*EO35+0.2379*CI35</f>
         <v>100.37289237499999</v>
       </c>
@@ -5168,7 +5164,7 @@
       <c r="C36" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D36" s="65">
+      <c r="D36" s="36">
         <f>0.4429*GQ36+0.2477*AA36+0.2386*CJ36+0.07079*CI36</f>
         <v>469.83887000000004</v>
       </c>
@@ -5199,7 +5195,7 @@
       <c r="C37" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D37" s="63" t="s">
+      <c r="D37" t="s">
         <v>401</v>
       </c>
       <c r="BC37">
@@ -5219,7 +5215,7 @@
       <c r="C38" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D38" s="63" t="s">
+      <c r="D38" t="s">
         <v>401</v>
       </c>
       <c r="BC38">
@@ -5239,7 +5235,7 @@
       <c r="C39" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="D39" t="s">
         <v>401</v>
       </c>
       <c r="BC39">
@@ -5259,7 +5255,7 @@
       <c r="C40" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D40" s="63" t="s">
+      <c r="D40" t="s">
         <v>708</v>
       </c>
       <c r="FT40" s="57"/>
@@ -5274,7 +5270,7 @@
       <c r="C41" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D41" s="63" t="s">
+      <c r="D41" t="s">
         <v>638</v>
       </c>
       <c r="BC41">
@@ -5292,7 +5288,7 @@
       <c r="C42" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D42" s="63" t="s">
+      <c r="D42" t="s">
         <v>635</v>
       </c>
       <c r="FT42" s="57"/>
@@ -5307,7 +5303,7 @@
       <c r="C43" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D43" s="63" t="s">
+      <c r="D43" t="s">
         <v>641</v>
       </c>
       <c r="FT43" s="57"/>
@@ -5322,7 +5318,7 @@
       <c r="C44" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D44" s="63" t="s">
+      <c r="D44" t="s">
         <v>636</v>
       </c>
       <c r="FT44" s="57"/>
@@ -5354,7 +5350,7 @@
       <c r="C46" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D46" s="63" t="s">
+      <c r="D46" t="s">
         <v>646</v>
       </c>
       <c r="FT46" s="57"/>
@@ -5369,7 +5365,7 @@
       <c r="C47" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="63" t="s">
+      <c r="D47" t="s">
         <v>639</v>
       </c>
       <c r="FT47" s="57">
@@ -5386,7 +5382,7 @@
       <c r="C48" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D48" s="66">
+      <c r="D48" s="63">
         <f>0.6941*AP48+0.2774*CI48+0.02849*J48</f>
         <v>72.171999999999997</v>
       </c>
@@ -5411,7 +5407,7 @@
       <c r="C49" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D49" s="63" t="s">
+      <c r="D49" t="s">
         <v>627</v>
       </c>
       <c r="FT49" s="57"/>
@@ -5426,7 +5422,7 @@
       <c r="C50" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D50" s="63" t="s">
+      <c r="D50" t="s">
         <v>318</v>
       </c>
       <c r="CO50" s="36">
@@ -5448,7 +5444,7 @@
       <c r="C51" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D51" s="63" t="s">
+      <c r="D51" t="s">
         <v>401</v>
       </c>
       <c r="BC51">
@@ -5468,7 +5464,7 @@
       <c r="C52" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D52" s="63" t="s">
+      <c r="D52" t="s">
         <v>397</v>
       </c>
       <c r="FP52">
@@ -5486,7 +5482,7 @@
       <c r="C53" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D53" s="63" t="s">
+      <c r="D53" t="s">
         <v>401</v>
       </c>
       <c r="FT53" s="57">
@@ -5503,7 +5499,7 @@
       <c r="C54" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D54" s="63" t="s">
+      <c r="D54" t="s">
         <v>401</v>
       </c>
       <c r="BC54">
@@ -5523,7 +5519,7 @@
       <c r="C55" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D55" s="63" t="s">
+      <c r="D55" t="s">
         <v>401</v>
       </c>
       <c r="FP55">
@@ -5543,7 +5539,7 @@
       <c r="C56" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D56" s="63" t="s">
+      <c r="D56" t="s">
         <v>632</v>
       </c>
       <c r="BC56">
@@ -5561,7 +5557,7 @@
       <c r="C57" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D57" s="63" t="s">
+      <c r="D57" t="s">
         <v>401</v>
       </c>
       <c r="BC57">
@@ -5620,7 +5616,7 @@
       <c r="C60" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D60" s="63" t="s">
+      <c r="D60" t="s">
         <v>401</v>
       </c>
       <c r="BC60">
@@ -5640,7 +5636,7 @@
       <c r="C61" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D61" s="67" t="s">
+      <c r="D61" s="2" t="s">
         <v>313</v>
       </c>
       <c r="CJ61">
@@ -5661,7 +5657,7 @@
       <c r="C62" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D62" s="65">
+      <c r="D62" s="36">
         <f>0.6712*FP62+0.3288*CO62</f>
         <v>74.023319999999998</v>
       </c>
@@ -5684,7 +5680,7 @@
       <c r="C63" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D63" s="63" t="s">
+      <c r="D63" t="s">
         <v>401</v>
       </c>
       <c r="BC63">
@@ -5722,7 +5718,7 @@
       <c r="C65" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D65" s="63" t="s">
+      <c r="D65" t="s">
         <v>629</v>
       </c>
       <c r="BC65">
@@ -5742,7 +5738,7 @@
       <c r="C66" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D66" s="63" t="s">
+      <c r="D66" t="s">
         <v>634</v>
       </c>
       <c r="BC66">
@@ -5760,7 +5756,7 @@
       <c r="C67" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D67" s="63" t="s">
+      <c r="D67" t="s">
         <v>640</v>
       </c>
       <c r="BC67">
@@ -5778,7 +5774,7 @@
       <c r="C68" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D68" s="63" t="s">
+      <c r="D68" t="s">
         <v>628</v>
       </c>
       <c r="BC68">
@@ -5798,7 +5794,7 @@
       <c r="C69" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D69" s="63" t="s">
+      <c r="D69" t="s">
         <v>734</v>
       </c>
       <c r="FT69" s="56"/>
@@ -5813,7 +5809,7 @@
       <c r="C70" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D70" s="63" t="s">
+      <c r="D70" t="s">
         <v>635</v>
       </c>
       <c r="BC70">
@@ -5870,7 +5866,7 @@
       <c r="C73" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D73" s="63" t="s">
+      <c r="D73" t="s">
         <v>401</v>
       </c>
       <c r="BC73">
@@ -5890,7 +5886,7 @@
       <c r="C74" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D74" s="63" t="s">
+      <c r="D74" t="s">
         <v>401</v>
       </c>
       <c r="BC74">
@@ -5910,7 +5906,7 @@
       <c r="C75" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D75" s="63" t="s">
+      <c r="D75" t="s">
         <v>401</v>
       </c>
       <c r="BC75">
@@ -5930,7 +5926,7 @@
       <c r="C76" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D76" s="67" t="s">
+      <c r="D76" s="2" t="s">
         <v>273</v>
       </c>
       <c r="AU76">
@@ -5949,7 +5945,7 @@
       <c r="C77" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D77" s="63" t="s">
+      <c r="D77" t="s">
         <v>401</v>
       </c>
       <c r="FT77" s="56">
@@ -5966,7 +5962,7 @@
       <c r="C78" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D78" s="63" t="s">
+      <c r="D78" t="s">
         <v>641</v>
       </c>
       <c r="FT78" s="56"/>
@@ -5996,7 +5992,7 @@
       <c r="C80" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D80" s="63" t="s">
+      <c r="D80" t="s">
         <v>401</v>
       </c>
       <c r="BC80">
@@ -6016,7 +6012,7 @@
       <c r="C81" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D81" s="63" t="s">
+      <c r="D81" t="s">
         <v>401</v>
       </c>
       <c r="FT81" s="56">
@@ -6033,7 +6029,7 @@
       <c r="C82" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D82" s="63" t="s">
+      <c r="D82" t="s">
         <v>634</v>
       </c>
       <c r="FT82" s="56"/>
@@ -6063,7 +6059,7 @@
       <c r="C84" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D84" s="63" t="s">
+      <c r="D84" t="s">
         <v>401</v>
       </c>
       <c r="BC84">
@@ -6083,7 +6079,7 @@
       <c r="C85" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D85" s="63" t="s">
+      <c r="D85" t="s">
         <v>401</v>
       </c>
       <c r="BC85">
@@ -6103,7 +6099,7 @@
       <c r="C86" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="D86" s="63" t="s">
+      <c r="D86" t="s">
         <v>401</v>
       </c>
       <c r="BC86">
@@ -6123,7 +6119,7 @@
       <c r="C87" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D87" s="63" t="s">
+      <c r="D87" t="s">
         <v>401</v>
       </c>
       <c r="FT87" s="56">
@@ -6196,7 +6192,7 @@
       <c r="C89" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D89" s="63" t="s">
+      <c r="D89" t="s">
         <v>401</v>
       </c>
       <c r="BC89">
@@ -6259,7 +6255,7 @@
       <c r="C91" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D91" s="63" t="s">
+      <c r="D91" t="s">
         <v>636</v>
       </c>
       <c r="BC91">
@@ -6331,7 +6327,7 @@
       <c r="C93" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D93" s="63" t="s">
+      <c r="D93" t="s">
         <v>401</v>
       </c>
       <c r="BC93">
@@ -6351,7 +6347,7 @@
       <c r="C94" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D94" s="63" t="s">
+      <c r="D94" t="s">
         <v>401</v>
       </c>
       <c r="BC94">
@@ -6371,7 +6367,7 @@
       <c r="C95" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D95" s="63" t="s">
+      <c r="D95" t="s">
         <v>401</v>
       </c>
       <c r="BC95">
@@ -6450,7 +6446,7 @@
       <c r="C98" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D98" s="63" t="s">
+      <c r="D98" t="s">
         <v>264</v>
       </c>
       <c r="AP98">
@@ -6468,7 +6464,7 @@
       <c r="C99" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D99" s="63" t="s">
+      <c r="D99" t="s">
         <v>641</v>
       </c>
       <c r="FT99" s="56"/>
@@ -6483,7 +6479,7 @@
       <c r="C100" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D100" s="63" t="s">
+      <c r="D100" t="s">
         <v>401</v>
       </c>
       <c r="BC100">
@@ -6503,7 +6499,7 @@
       <c r="C101" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D101" s="63" t="s">
+      <c r="D101" t="s">
         <v>748</v>
       </c>
       <c r="BC101">
@@ -6521,7 +6517,7 @@
       <c r="C102" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D102" s="63" t="s">
+      <c r="D102" t="s">
         <v>401</v>
       </c>
       <c r="BC102">
@@ -6541,7 +6537,7 @@
       <c r="C103" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D103" s="63" t="s">
+      <c r="D103" t="s">
         <v>627</v>
       </c>
       <c r="FT103" s="56"/>
@@ -6556,7 +6552,7 @@
       <c r="C104" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D104" s="63" t="s">
+      <c r="D104" t="s">
         <v>642</v>
       </c>
       <c r="FT104" s="56"/>
@@ -6571,7 +6567,7 @@
       <c r="C105" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D105" s="63" t="s">
+      <c r="D105" t="s">
         <v>642</v>
       </c>
       <c r="FT105" s="56"/>
@@ -6586,7 +6582,7 @@
       <c r="C106" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D106" s="63" t="s">
+      <c r="D106" t="s">
         <v>401</v>
       </c>
       <c r="BC106">
@@ -6606,7 +6602,7 @@
       <c r="C107" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D107" s="63" t="s">
+      <c r="D107" t="s">
         <v>401</v>
       </c>
       <c r="BC107">
@@ -6626,7 +6622,7 @@
       <c r="C108" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D108" s="63" t="s">
+      <c r="D108" t="s">
         <v>401</v>
       </c>
       <c r="BC108">
@@ -6696,11 +6692,11 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" s="37" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
@@ -7457,6 +7453,10 @@
       <c r="C65" s="2" t="s">
         <v>111</v>
       </c>
+      <c r="D65">
+        <f>0.021/6.25</f>
+        <v>3.3600000000000001E-3</v>
+      </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
@@ -7577,6 +7577,10 @@
       </c>
       <c r="C75" s="2" t="s">
         <v>111</v>
+      </c>
+      <c r="D75">
+        <f>0.021/6.25</f>
+        <v>3.3600000000000001E-3</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
@@ -7986,9 +7990,12 @@
       <c r="C115" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{C879ADC7-81D3-4EBF-86D2-61BB228F73CB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -11538,23 +11545,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x010100A603BB68AE5C0F4C908E70EB4D1DDDC3" ma:contentTypeVersion="15" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="bc1901b771652496ef02f4cbdf878f9e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95" xmlns:ns4="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c61e44642a1e9e2aad865b2f0b39e8f" ns3:_="" ns4:_="">
     <xsd:import namespace="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95"/>
@@ -11789,25 +11779,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27BF0A1B-B2BC-4159-BD4C-213AA0853490}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11824,4 +11813,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
New N fertiliser file
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{916EBC08-63FA-4880-A697-77B5FD265A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46413638-2373-479F-89B1-85401360A5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -123,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2150" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2160" uniqueCount="753">
   <si>
     <t>Crops</t>
   </si>
@@ -2466,6 +2466,12 @@
   </si>
   <si>
     <t>Approx cantaloupes</t>
+  </si>
+  <si>
+    <t>Yara (2018)</t>
+  </si>
+  <si>
+    <t>Yara (2018). Gödslingsråd. https://www.yara.se/contentassets/b2d039536ac14ce382a98e12dd92282e/yar0050_godslingsradet_2018_okt.pdf</t>
   </si>
 </sst>
 </file>
@@ -2689,7 +2695,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2834,6 +2840,10 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Hyperlink" xfId="11" xr:uid="{27B946F3-5790-4F7E-8391-6BBF48B2CC3B}"/>
@@ -3341,7 +3351,7 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A2:GT115"/>
+  <dimension ref="A2:GT118"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="32.90625" customWidth="1"/>
@@ -4888,7 +4898,10 @@
       <c r="BC21">
         <v>0</v>
       </c>
-      <c r="FT21" s="57"/>
+      <c r="FT21" s="64">
+        <f>AVERAGE(30,40)</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="22" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
@@ -4906,8 +4919,9 @@
       <c r="BC22">
         <v>215</v>
       </c>
-      <c r="FT22" s="57">
-        <v>150</v>
+      <c r="FT22" s="64">
+        <f>AVERAGE(180,250)</f>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:176" x14ac:dyDescent="0.35">
@@ -4940,8 +4954,9 @@
       <c r="BC24">
         <v>285</v>
       </c>
-      <c r="FT24" s="56">
-        <v>200.00035800590709</v>
+      <c r="FT24" s="65">
+        <f>AVERAGE(180,300)</f>
+        <v>240</v>
       </c>
     </row>
     <row r="25" spans="1:176" x14ac:dyDescent="0.35">
@@ -4977,8 +4992,9 @@
       <c r="BC26">
         <v>400</v>
       </c>
-      <c r="FT26" s="57">
-        <v>83</v>
+      <c r="FT26" s="64">
+        <f>AVERAGE(60,150)</f>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:176" x14ac:dyDescent="0.35">
@@ -5016,8 +5032,9 @@
         <v>255</v>
       </c>
       <c r="FP28" s="28"/>
-      <c r="FT28" s="57">
-        <v>220</v>
+      <c r="FT28" s="64">
+        <f>AVERAGE(220, 280)</f>
+        <v>250</v>
       </c>
     </row>
     <row r="29" spans="1:176" x14ac:dyDescent="0.35">
@@ -5033,8 +5050,9 @@
       <c r="D29" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="FT29" s="56">
-        <v>192.00000000000003</v>
+      <c r="FT29" s="65">
+        <f>AVERAGE(FT28,FT22)</f>
+        <v>232.5</v>
       </c>
     </row>
     <row r="30" spans="1:176" x14ac:dyDescent="0.35">
@@ -5450,8 +5468,9 @@
       <c r="BC51">
         <v>225</v>
       </c>
-      <c r="FT51" s="57">
-        <v>219.9992474773388</v>
+      <c r="FT51" s="64">
+        <f>AVERAGE(180,220)</f>
+        <v>200</v>
       </c>
     </row>
     <row r="52" spans="1:176" x14ac:dyDescent="0.35">
@@ -5505,8 +5524,9 @@
       <c r="BC54">
         <v>150</v>
       </c>
-      <c r="FT54" s="57">
-        <v>103.99894409543754</v>
+      <c r="FT54" s="64">
+        <f>AVERAGE(100,150)</f>
+        <v>125</v>
       </c>
     </row>
     <row r="55" spans="1:176" x14ac:dyDescent="0.35">
@@ -5912,8 +5932,9 @@
       <c r="BC75">
         <v>0</v>
       </c>
-      <c r="FT75" s="56">
-        <v>0</v>
+      <c r="FT75" s="65">
+        <f>AVERAGE(30,40)</f>
+        <v>35</v>
       </c>
     </row>
     <row r="76" spans="1:176" x14ac:dyDescent="0.35">
@@ -6015,8 +6036,9 @@
       <c r="D81" t="s">
         <v>401</v>
       </c>
-      <c r="FT81" s="56">
-        <v>17.999882715781244</v>
+      <c r="FT81" s="65">
+        <f>AVERAGE(90,170)</f>
+        <v>130</v>
       </c>
     </row>
     <row r="82" spans="1:199" x14ac:dyDescent="0.35">
@@ -6652,20 +6674,23 @@
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:181" x14ac:dyDescent="0.35">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:181" x14ac:dyDescent="0.35">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:181" x14ac:dyDescent="0.35">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
+    </row>
+    <row r="118" spans="1:181" x14ac:dyDescent="0.35">
+      <c r="FY118" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9446,7 +9471,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="17" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -9466,7 +9491,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="18" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -9486,7 +9511,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="19" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -9502,7 +9527,7 @@
       <c r="BC19" s="44"/>
       <c r="BD19" s="44"/>
     </row>
-    <row r="20" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -9522,7 +9547,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="21" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -9541,8 +9566,11 @@
       <c r="BD21" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="22" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT21" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -9561,8 +9589,11 @@
       <c r="BD22" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="23" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT22" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -9578,7 +9609,7 @@
       <c r="BC23" s="44"/>
       <c r="BD23" s="44"/>
     </row>
-    <row r="24" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -9597,8 +9628,11 @@
       <c r="BD24" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="25" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT24" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -9617,7 +9651,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="26" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -9636,8 +9670,11 @@
       <c r="BD26" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="27" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT26" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -9656,7 +9693,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="28" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -9675,8 +9712,11 @@
       <c r="BD28" s="41" t="s">
         <v>676</v>
       </c>
-    </row>
-    <row r="29" spans="1:172" x14ac:dyDescent="0.35">
+      <c r="FT28" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -9692,7 +9732,7 @@
       <c r="BC29" s="39"/>
       <c r="BD29" s="39"/>
     </row>
-    <row r="30" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -9709,7 +9749,7 @@
       <c r="BC30" s="47"/>
       <c r="BD30" s="47"/>
     </row>
-    <row r="31" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -9725,7 +9765,7 @@
       <c r="BC31" s="47"/>
       <c r="BD31" s="47"/>
     </row>
-    <row r="32" spans="1:172" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -10103,6 +10143,9 @@
       <c r="BD51" s="41" t="s">
         <v>676</v>
       </c>
+      <c r="FT51" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="52" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
@@ -10161,6 +10204,9 @@
       <c r="BD54" s="41" t="s">
         <v>676</v>
       </c>
+      <c r="FT54" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="55" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
@@ -10572,6 +10618,9 @@
       <c r="BD75" s="41" t="s">
         <v>676</v>
       </c>
+      <c r="FT75" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="76" spans="1:176" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
@@ -10675,6 +10724,9 @@
       </c>
       <c r="BC81" s="39"/>
       <c r="BD81" s="39"/>
+      <c r="FT81" t="s">
+        <v>751</v>
+      </c>
     </row>
     <row r="82" spans="1:199" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
@@ -11443,7 +11495,9 @@
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A12" s="5"/>
+      <c r="A12" s="5" t="s">
+        <v>752</v>
+      </c>
       <c r="S12" s="9"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update footprints data files (output)
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
+++ b/data-preprocessing/rpc-footprints/1 - Crops/N fertiliser.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr filterPrivacy="1" updateLinks="never" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46413638-2373-479F-89B1-85401360A5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDAC5170-65A7-F643-8104-E0CEAE6D429E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29240" windowHeight="18380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="117" r:id="rId1"/>
@@ -36,7 +36,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -47,7 +46,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>Författare</author>
+    <author>Author</author>
   </authors>
   <commentList>
     <comment ref="D56" authorId="0" shapeId="0" xr:uid="{1D56F74A-6B95-468C-8D09-3316D2AD7FD4}">
@@ -60,7 +59,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Författare:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -81,8 +80,7 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>Författare</author>
-    <author>tc={A44E80FC-CA83-4236-ACE7-C34F982CF278}</author>
+    <author>Author</author>
   </authors>
   <commentList>
     <comment ref="D12" authorId="0" shapeId="0" xr:uid="{05B678CA-DD0D-4DAD-9149-002738F80FF2}">
@@ -95,7 +93,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Författare:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -110,12 +108,21 @@
         </r>
       </text>
     </comment>
-    <comment ref="AU34" authorId="1" shapeId="0" xr:uid="{A44E80FC-CA83-4236-ACE7-C34F982CF278}">
+    <comment ref="AU34" authorId="0" shapeId="0" xr:uid="{A44E80FC-CA83-4236-ACE7-C34F982CF278}">
       <text>
-        <t>[Trådad kommentar]
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>[Trådad kommentar]
 I din version av Excel kan du läsa den här trådade kommentaren, men eventuella ändringar i den tas bort om filen öppnas i en senare version av Excel. Läs mer: https://go.microsoft.com/fwlink/?linkid=870924
 Kommentar:
     Sebastian Castro-Tanzi, Thomas Dietsch, Natalia Urena, Lucia Vindas, Mark Chandler.  Analysis of management and site factors to improve the sustainability of smallholder coffee production in Tarrazú, Costa Rica, Agriculture, Ecosystems &amp; Environment, Volume 155, 2012, p 172-181</t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -123,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2160" uniqueCount="753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2161" uniqueCount="753">
   <si>
     <t>Crops</t>
   </si>
@@ -2649,7 +2656,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2668,6 +2675,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2678,7 +2691,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="13">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0"/>
@@ -2692,10 +2705,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2783,13 +2795,13 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="20" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="20" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="21" fillId="0" borderId="0" xfId="12" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="21" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2798,7 +2810,7 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="20" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="20" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="21" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2807,7 +2819,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="12" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -2844,14 +2856,14 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="13">
-    <cellStyle name="Hyperlink" xfId="11" xr:uid="{27B946F3-5790-4F7E-8391-6BBF48B2CC3B}"/>
-    <cellStyle name="Hyperlänk" xfId="10" builtinId="8"/>
+  <cellStyles count="12">
+    <cellStyle name="Hyperlink" xfId="10" xr:uid="{27B946F3-5790-4F7E-8391-6BBF48B2CC3B}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 2 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2 3" xfId="12" xr:uid="{73C79919-7B37-44A4-B3CF-0A4A3A6DB9B5}"/>
+    <cellStyle name="Normal 2 3" xfId="11" xr:uid="{73C79919-7B37-44A4-B3CF-0A4A3A6DB9B5}"/>
     <cellStyle name="Normal 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Normal 4" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Normal 5" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
@@ -3153,31 +3165,31 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A2:G22"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="27.26953125" customWidth="1"/>
-    <col min="3" max="3" width="13.08984375" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>663</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>664</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="31"/>
     </row>
-    <row r="8" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
         <v>1</v>
       </c>
@@ -3191,7 +3203,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -3208,7 +3220,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -3225,7 +3237,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -3242,7 +3254,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -3259,7 +3271,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>76</v>
       </c>
@@ -3276,7 +3288,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>58</v>
       </c>
@@ -3290,7 +3302,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
         <v>658</v>
       </c>
@@ -3304,7 +3316,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>654</v>
       </c>
@@ -3319,7 +3331,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>657</v>
       </c>
@@ -3334,7 +3346,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="19"/>
     </row>
   </sheetData>
@@ -3352,22 +3364,22 @@
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A2:GT118"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="32.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" customWidth="1"/>
-    <col min="5" max="175" width="5.6328125" customWidth="1"/>
-    <col min="176" max="176" width="5.6328125" style="1" customWidth="1"/>
-    <col min="177" max="202" width="5.6328125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
+    <col min="5" max="175" width="5.6640625" customWidth="1"/>
+    <col min="176" max="176" width="5.6640625" style="1" customWidth="1"/>
+    <col min="177" max="202" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:202" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:202" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
@@ -3968,7 +3980,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="5" spans="1:202" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:202" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>1</v>
       </c>
@@ -4576,7 +4588,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="6" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -4607,7 +4619,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="7" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -4625,7 +4637,7 @@
       </c>
       <c r="FT7" s="56"/>
     </row>
-    <row r="8" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -4645,7 +4657,7 @@
         <v>41.000996934136801</v>
       </c>
     </row>
-    <row r="9" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -4660,7 +4672,7 @@
       </c>
       <c r="FT9" s="56"/>
     </row>
-    <row r="10" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -4678,7 +4690,7 @@
       </c>
       <c r="FT10" s="56"/>
     </row>
-    <row r="11" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -4698,7 +4710,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -4718,7 +4730,7 @@
       </c>
       <c r="FT12" s="56"/>
     </row>
-    <row r="13" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -4748,7 +4760,7 @@
       </c>
       <c r="FT13" s="56"/>
     </row>
-    <row r="14" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -4768,7 +4780,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -4788,7 +4800,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -4809,7 +4821,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -4829,7 +4841,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -4847,7 +4859,7 @@
       </c>
       <c r="FT18" s="57"/>
     </row>
-    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -4862,7 +4874,7 @@
       </c>
       <c r="FT19" s="56"/>
     </row>
-    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -4882,7 +4894,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -4903,7 +4915,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -4924,7 +4936,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -4938,7 +4950,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -4959,7 +4971,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -4976,7 +4988,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -4997,7 +5009,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -5015,7 +5027,7 @@
         <v>289.51785714285717</v>
       </c>
     </row>
-    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -5037,7 +5049,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -5055,7 +5067,7 @@
         <v>232.5</v>
       </c>
     </row>
-    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -5071,7 +5083,7 @@
       <c r="M30" s="28"/>
       <c r="FT30" s="57"/>
     </row>
-    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -5086,7 +5098,7 @@
       </c>
       <c r="FT31" s="57"/>
     </row>
-    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -5101,7 +5113,7 @@
       </c>
       <c r="FT32" s="56"/>
     </row>
-    <row r="33" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -5119,7 +5131,7 @@
       </c>
       <c r="FT33" s="56"/>
     </row>
-    <row r="34" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -5144,7 +5156,7 @@
       </c>
       <c r="FT34" s="56"/>
     </row>
-    <row r="35" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -5172,7 +5184,7 @@
       </c>
       <c r="FT35" s="56"/>
     </row>
-    <row r="36" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -5203,7 +5215,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="37" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -5223,7 +5235,7 @@
         <v>1451.4258</v>
       </c>
     </row>
-    <row r="38" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -5243,7 +5255,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -5263,7 +5275,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -5278,7 +5290,7 @@
       </c>
       <c r="FT40" s="57"/>
     </row>
-    <row r="41" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -5296,7 +5308,7 @@
       </c>
       <c r="FT41" s="57"/>
     </row>
-    <row r="42" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -5311,7 +5323,7 @@
       </c>
       <c r="FT42" s="57"/>
     </row>
-    <row r="43" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -5326,7 +5338,7 @@
       </c>
       <c r="FT43" s="57"/>
     </row>
-    <row r="44" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -5341,7 +5353,7 @@
       </c>
       <c r="FT44" s="57"/>
     </row>
-    <row r="45" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -5358,7 +5370,7 @@
         <v>6.2508461827754793</v>
       </c>
     </row>
-    <row r="46" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -5373,7 +5385,7 @@
       </c>
       <c r="FT46" s="57"/>
     </row>
-    <row r="47" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -5390,7 +5402,7 @@
         <v>11.387434554973822</v>
       </c>
     </row>
-    <row r="48" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -5415,7 +5427,7 @@
       </c>
       <c r="FT48" s="57"/>
     </row>
-    <row r="49" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -5430,7 +5442,7 @@
       </c>
       <c r="FT49" s="57"/>
     </row>
-    <row r="50" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -5452,7 +5464,7 @@
       </c>
       <c r="FT50" s="57"/>
     </row>
-    <row r="51" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -5473,7 +5485,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="52" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -5491,7 +5503,7 @@
       </c>
       <c r="FT52" s="57"/>
     </row>
-    <row r="53" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -5508,7 +5520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -5529,7 +5541,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="55" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -5549,7 +5561,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -5567,7 +5579,7 @@
       </c>
       <c r="FT56" s="57"/>
     </row>
-    <row r="57" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -5587,7 +5599,7 @@
         <v>131.99700453857793</v>
       </c>
     </row>
-    <row r="58" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -5605,7 +5617,7 @@
       </c>
       <c r="FT58" s="57"/>
     </row>
-    <row r="59" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -5626,7 +5638,7 @@
       </c>
       <c r="FT59" s="57"/>
     </row>
-    <row r="60" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
@@ -5646,7 +5658,7 @@
         <v>70.992046843177178</v>
       </c>
     </row>
-    <row r="61" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
@@ -5667,7 +5679,7 @@
       </c>
       <c r="FT61" s="56"/>
     </row>
-    <row r="62" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -5690,7 +5702,7 @@
       </c>
       <c r="FT62" s="56"/>
     </row>
-    <row r="63" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
@@ -5710,7 +5722,7 @@
         <v>143.99874345549739</v>
       </c>
     </row>
-    <row r="64" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
@@ -5728,7 +5740,7 @@
       </c>
       <c r="FT64" s="56"/>
     </row>
-    <row r="65" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
@@ -5748,7 +5760,7 @@
         <v>2.0001956181533647</v>
       </c>
     </row>
-    <row r="66" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
@@ -5766,7 +5778,7 @@
       </c>
       <c r="FT66" s="56"/>
     </row>
-    <row r="67" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
@@ -5784,7 +5796,7 @@
       </c>
       <c r="FT67" s="56"/>
     </row>
-    <row r="68" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
@@ -5804,7 +5816,7 @@
         <v>1.9994986631016041</v>
       </c>
     </row>
-    <row r="69" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -5819,7 +5831,7 @@
       </c>
       <c r="FT69" s="56"/>
     </row>
-    <row r="70" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -5839,7 +5851,7 @@
         <v>131.99427061709758</v>
       </c>
     </row>
-    <row r="71" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -5858,7 +5870,7 @@
       </c>
       <c r="FT71" s="56"/>
     </row>
-    <row r="72" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -5876,7 +5888,7 @@
       </c>
       <c r="FT72" s="56"/>
     </row>
-    <row r="73" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -5896,7 +5908,7 @@
         <v>48.001155234657041</v>
       </c>
     </row>
-    <row r="74" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -5916,7 +5928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
@@ -5937,7 +5949,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="76" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
@@ -5956,7 +5968,7 @@
       </c>
       <c r="FT76" s="56"/>
     </row>
-    <row r="77" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
@@ -5973,7 +5985,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="78" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
@@ -5988,7 +6000,7 @@
       </c>
       <c r="FT78" s="56"/>
     </row>
-    <row r="79" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -6003,7 +6015,7 @@
       </c>
       <c r="FT79" s="56"/>
     </row>
-    <row r="80" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
@@ -6023,7 +6035,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="81" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
@@ -6034,6 +6046,9 @@
         <v>111</v>
       </c>
       <c r="D81" t="s">
+        <v>401</v>
+      </c>
+      <c r="FP81" s="66" t="s">
         <v>401</v>
       </c>
       <c r="FT81" s="65">
@@ -6041,7 +6056,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="82" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
@@ -6056,7 +6071,7 @@
       </c>
       <c r="FT82" s="56"/>
     </row>
-    <row r="83" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
@@ -6071,7 +6086,7 @@
       </c>
       <c r="FT83" s="56"/>
     </row>
-    <row r="84" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
@@ -6091,7 +6106,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="85" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
@@ -6111,7 +6126,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="86" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
@@ -6131,7 +6146,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="87" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
@@ -6148,7 +6163,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="88" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
@@ -6204,7 +6219,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="89" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
@@ -6224,7 +6239,7 @@
         <v>95.003821656050945</v>
       </c>
     </row>
-    <row r="90" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
@@ -6267,7 +6282,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="91" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
@@ -6287,7 +6302,7 @@
         <v>99.990651635963701</v>
       </c>
     </row>
-    <row r="92" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
@@ -6339,7 +6354,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
@@ -6359,7 +6374,7 @@
         <v>44.998221845893312</v>
       </c>
     </row>
-    <row r="94" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
@@ -6379,7 +6394,7 @@
         <v>32.999338097028954</v>
       </c>
     </row>
-    <row r="95" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
@@ -6399,7 +6414,7 @@
         <v>104.9996533509409</v>
       </c>
     </row>
-    <row r="96" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
@@ -6418,7 +6433,7 @@
       </c>
       <c r="FT96" s="56"/>
     </row>
-    <row r="97" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
@@ -6458,7 +6473,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="98" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
@@ -6476,7 +6491,7 @@
       </c>
       <c r="FT98" s="56"/>
     </row>
-    <row r="99" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>98</v>
       </c>
@@ -6491,7 +6506,7 @@
       </c>
       <c r="FT99" s="56"/>
     </row>
-    <row r="100" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>99</v>
       </c>
@@ -6511,7 +6526,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="101" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>100</v>
       </c>
@@ -6529,7 +6544,7 @@
       </c>
       <c r="FT101" s="56"/>
     </row>
-    <row r="102" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>101</v>
       </c>
@@ -6549,7 +6564,7 @@
         <v>105.99222303741747</v>
       </c>
     </row>
-    <row r="103" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>102</v>
       </c>
@@ -6564,7 +6579,7 @@
       </c>
       <c r="FT103" s="56"/>
     </row>
-    <row r="104" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
         <v>103</v>
       </c>
@@ -6579,7 +6594,7 @@
       </c>
       <c r="FT104" s="56"/>
     </row>
-    <row r="105" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>104</v>
       </c>
@@ -6594,7 +6609,7 @@
       </c>
       <c r="FT105" s="56"/>
     </row>
-    <row r="106" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>105</v>
       </c>
@@ -6614,7 +6629,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="107" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -6634,7 +6649,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="108" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>107</v>
       </c>
@@ -6654,42 +6669,42 @@
         <v>159</v>
       </c>
     </row>
-    <row r="109" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:181" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:181" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:181" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:181" x14ac:dyDescent="0.2">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:181" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:181" x14ac:dyDescent="0.2">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
     </row>
-    <row r="118" spans="1:181" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:181" x14ac:dyDescent="0.2">
       <c r="FY118" s="19"/>
     </row>
   </sheetData>
@@ -6704,31 +6719,31 @@
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A2:D115"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="32.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="37" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>1</v>
       </c>
@@ -6742,7 +6757,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -6754,7 +6769,7 @@
       </c>
       <c r="D6" s="38"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -6766,7 +6781,7 @@
       </c>
       <c r="D7" s="53"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -6778,7 +6793,7 @@
       </c>
       <c r="D8" s="19"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -6790,7 +6805,7 @@
       </c>
       <c r="D9" s="19"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -6802,7 +6817,7 @@
       </c>
       <c r="D10" s="19"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -6814,7 +6829,7 @@
       </c>
       <c r="D11" s="19"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -6826,7 +6841,7 @@
       </c>
       <c r="D12" s="53"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -6838,7 +6853,7 @@
       </c>
       <c r="D13" s="38"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -6850,7 +6865,7 @@
       </c>
       <c r="D14" s="19"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -6862,7 +6877,7 @@
       </c>
       <c r="D15" s="19"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -6874,7 +6889,7 @@
       </c>
       <c r="D16" s="19"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -6889,7 +6904,7 @@
         <v>3.5200000000000002E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -6901,7 +6916,7 @@
       </c>
       <c r="D18" s="19"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -6913,7 +6928,7 @@
       </c>
       <c r="D19" s="19"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -6928,7 +6943,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -6943,7 +6958,7 @@
         <v>1.44E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -6955,7 +6970,7 @@
       </c>
       <c r="D22" s="19"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -6967,7 +6982,7 @@
       </c>
       <c r="D23" s="19"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -6979,7 +6994,7 @@
       </c>
       <c r="D24" s="19"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -6991,7 +7006,7 @@
       </c>
       <c r="D25" s="19"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -7003,7 +7018,7 @@
       </c>
       <c r="D26" s="19"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -7015,7 +7030,7 @@
       </c>
       <c r="D27" s="19"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -7027,7 +7042,7 @@
       </c>
       <c r="D28" s="53"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -7039,7 +7054,7 @@
       </c>
       <c r="D29" s="53"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -7051,7 +7066,7 @@
       </c>
       <c r="D30" s="19"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -7063,7 +7078,7 @@
       </c>
       <c r="D31" s="19"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -7078,7 +7093,7 @@
         <v>3.0079999999999999E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -7090,7 +7105,7 @@
       </c>
       <c r="D33" s="19"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -7102,7 +7117,7 @@
       </c>
       <c r="D34" s="38"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -7114,7 +7129,7 @@
       </c>
       <c r="D35" s="38"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -7126,7 +7141,7 @@
       </c>
       <c r="D36" s="38"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -7138,7 +7153,7 @@
       </c>
       <c r="D37" s="19"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -7150,7 +7165,7 @@
       </c>
       <c r="D38" s="19"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -7162,7 +7177,7 @@
       </c>
       <c r="D39" s="19"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -7174,7 +7189,7 @@
       </c>
       <c r="D40" s="19"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -7186,7 +7201,7 @@
       </c>
       <c r="D41" s="19"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -7198,7 +7213,7 @@
       </c>
       <c r="D42" s="19"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -7210,7 +7225,7 @@
       </c>
       <c r="D43" s="19"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -7222,7 +7237,7 @@
       </c>
       <c r="D44" s="19"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -7234,7 +7249,7 @@
       </c>
       <c r="D45" s="53"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -7246,7 +7261,7 @@
       </c>
       <c r="D46" s="19"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -7258,7 +7273,7 @@
       </c>
       <c r="D47" s="19"/>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -7270,7 +7285,7 @@
       </c>
       <c r="D48" s="59"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -7282,7 +7297,7 @@
       </c>
       <c r="D49" s="19"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -7294,7 +7309,7 @@
       </c>
       <c r="D50" s="19"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -7306,7 +7321,7 @@
       </c>
       <c r="D51" s="19"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -7318,7 +7333,7 @@
       </c>
       <c r="D52" s="19"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -7333,7 +7348,7 @@
         <v>3.9039999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -7345,7 +7360,7 @@
       </c>
       <c r="D54" s="19"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -7357,7 +7372,7 @@
       </c>
       <c r="D55" s="19"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -7372,7 +7387,7 @@
         <v>3.5200000000000002E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -7384,7 +7399,7 @@
       </c>
       <c r="D57" s="19"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -7396,7 +7411,7 @@
       </c>
       <c r="D58" s="53"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -7408,7 +7423,7 @@
       </c>
       <c r="D59" s="53"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
@@ -7420,7 +7435,7 @@
       </c>
       <c r="D60" s="19"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
@@ -7432,7 +7447,7 @@
       </c>
       <c r="D61" s="25"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -7444,7 +7459,7 @@
       </c>
       <c r="D62" s="38"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
@@ -7456,7 +7471,7 @@
       </c>
       <c r="D63" s="19"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
@@ -7468,7 +7483,7 @@
       </c>
       <c r="D64" s="53"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
@@ -7483,7 +7498,7 @@
         <v>3.3600000000000001E-3</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
@@ -7494,7 +7509,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
@@ -7505,7 +7520,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
@@ -7520,7 +7535,7 @@
         <v>3.5200000000000002E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -7531,7 +7546,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -7542,7 +7557,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -7554,7 +7569,7 @@
       </c>
       <c r="D71" s="53"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -7566,7 +7581,7 @@
       </c>
       <c r="D72" s="53"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -7578,7 +7593,7 @@
       </c>
       <c r="D73" s="19"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -7593,7 +7608,7 @@
         <v>3.44E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
@@ -7608,7 +7623,7 @@
         <v>3.3600000000000001E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
@@ -7620,7 +7635,7 @@
       </c>
       <c r="D76" s="2"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
@@ -7631,7 +7646,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
@@ -7642,7 +7657,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -7654,7 +7669,7 @@
       </c>
       <c r="D79" s="1"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
@@ -7665,7 +7680,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
@@ -7676,7 +7691,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
@@ -7687,7 +7702,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
@@ -7699,7 +7714,7 @@
       </c>
       <c r="D83" s="28"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
@@ -7710,7 +7725,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
@@ -7721,7 +7736,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
@@ -7732,7 +7747,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
@@ -7743,7 +7758,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
@@ -7755,7 +7770,7 @@
       </c>
       <c r="D88" s="1"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
@@ -7766,7 +7781,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
@@ -7777,7 +7792,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
@@ -7788,7 +7803,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
@@ -7803,7 +7818,7 @@
         <v>6.0479999999999999E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
@@ -7814,7 +7829,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
@@ -7825,7 +7840,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
@@ -7836,7 +7851,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
@@ -7847,7 +7862,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
@@ -7858,7 +7873,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
@@ -7869,7 +7884,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>98</v>
       </c>
@@ -7880,7 +7895,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>99</v>
       </c>
@@ -7891,7 +7906,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>100</v>
       </c>
@@ -7902,7 +7917,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>101</v>
       </c>
@@ -7913,7 +7928,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>102</v>
       </c>
@@ -7924,7 +7939,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
         <v>103</v>
       </c>
@@ -7935,7 +7950,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>104</v>
       </c>
@@ -7946,7 +7961,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>105</v>
       </c>
@@ -7957,7 +7972,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -7968,7 +7983,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>107</v>
       </c>
@@ -7979,37 +7994,37 @@
         <v>122</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -8030,20 +8045,20 @@
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A2:GT115"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="32.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.36328125" customWidth="1"/>
-    <col min="4" max="4" width="14.90625" customWidth="1"/>
-    <col min="5" max="202" width="5.6328125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="202" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:202" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:202" ht="19" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:202" ht="78.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
@@ -8644,7 +8659,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="5" spans="1:202" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:202" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>1</v>
       </c>
@@ -9252,7 +9267,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="6" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -9275,7 +9290,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="7" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -9292,7 +9307,7 @@
       <c r="BC7" s="39"/>
       <c r="BD7" s="39"/>
     </row>
-    <row r="8" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -9312,7 +9327,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="9" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -9328,7 +9343,7 @@
       <c r="BC9" s="39"/>
       <c r="BD9" s="39"/>
     </row>
-    <row r="10" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -9348,7 +9363,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="11" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -9368,7 +9383,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="12" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -9387,7 +9402,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -9415,7 +9430,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="14" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -9431,7 +9446,7 @@
       <c r="BC14" s="40"/>
       <c r="BD14" s="41"/>
     </row>
-    <row r="15" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -9451,7 +9466,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="16" spans="1:202" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:202" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -9471,7 +9486,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="17" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -9491,7 +9506,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="18" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -9511,7 +9526,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="19" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -9527,7 +9542,7 @@
       <c r="BC19" s="44"/>
       <c r="BD19" s="44"/>
     </row>
-    <row r="20" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -9547,7 +9562,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="21" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -9570,7 +9585,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="22" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -9593,7 +9608,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="23" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -9609,7 +9624,7 @@
       <c r="BC23" s="44"/>
       <c r="BD23" s="44"/>
     </row>
-    <row r="24" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -9632,7 +9647,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="25" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -9651,7 +9666,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="26" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -9674,7 +9689,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="27" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -9693,7 +9708,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="28" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -9716,7 +9731,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="29" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -9732,7 +9747,7 @@
       <c r="BC29" s="39"/>
       <c r="BD29" s="39"/>
     </row>
-    <row r="30" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -9749,7 +9764,7 @@
       <c r="BC30" s="47"/>
       <c r="BD30" s="47"/>
     </row>
-    <row r="31" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -9765,7 +9780,7 @@
       <c r="BC31" s="47"/>
       <c r="BD31" s="47"/>
     </row>
-    <row r="32" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -9781,7 +9796,7 @@
       <c r="BC32" s="39"/>
       <c r="BD32" s="39"/>
     </row>
-    <row r="33" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -9800,7 +9815,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="34" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -9828,7 +9843,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="35" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -9844,7 +9859,7 @@
       <c r="BC35" s="48"/>
       <c r="BD35" s="48"/>
     </row>
-    <row r="36" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -9872,7 +9887,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="37" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -9892,7 +9907,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="38" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -9912,7 +9927,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="39" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -9932,7 +9947,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="40" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -9948,7 +9963,7 @@
       <c r="BC40" s="39"/>
       <c r="BD40" s="39"/>
     </row>
-    <row r="41" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -9968,7 +9983,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="42" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -9984,7 +9999,7 @@
       <c r="BC42" s="39"/>
       <c r="BD42" s="39"/>
     </row>
-    <row r="43" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -10000,7 +10015,7 @@
       <c r="BC43" s="42"/>
       <c r="BD43" s="42"/>
     </row>
-    <row r="44" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -10016,7 +10031,7 @@
       <c r="BC44" s="39"/>
       <c r="BD44" s="39"/>
     </row>
-    <row r="45" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -10032,7 +10047,7 @@
       <c r="BC45" s="39"/>
       <c r="BD45" s="39"/>
     </row>
-    <row r="46" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -10048,7 +10063,7 @@
       <c r="BC46" s="48"/>
       <c r="BD46" s="48"/>
     </row>
-    <row r="47" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -10064,7 +10079,7 @@
       <c r="BC47" s="47"/>
       <c r="BD47" s="47"/>
     </row>
-    <row r="48" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -10089,7 +10104,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="49" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -10105,7 +10120,7 @@
       <c r="BC49" s="47"/>
       <c r="BD49" s="47"/>
     </row>
-    <row r="50" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -10124,7 +10139,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="51" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -10147,7 +10162,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="52" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -10166,7 +10181,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="53" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -10185,7 +10200,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="54" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -10208,7 +10223,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="55" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -10224,7 +10239,7 @@
       <c r="BC55" s="47"/>
       <c r="BD55" s="47"/>
     </row>
-    <row r="56" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -10244,7 +10259,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="57" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -10264,7 +10279,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="58" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -10283,7 +10298,7 @@
       <c r="BC58" s="48"/>
       <c r="BD58" s="48"/>
     </row>
-    <row r="59" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -10302,7 +10317,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="60" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
@@ -10322,7 +10337,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="61" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
@@ -10341,7 +10356,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="62" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
@@ -10363,7 +10378,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="63" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
@@ -10383,7 +10398,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="64" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
@@ -10402,7 +10417,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="65" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
@@ -10422,7 +10437,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="66" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
@@ -10442,7 +10457,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="67" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
@@ -10462,7 +10477,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="68" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
@@ -10482,7 +10497,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="69" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -10498,7 +10513,7 @@
       <c r="BC69" s="39"/>
       <c r="BD69" s="39"/>
     </row>
-    <row r="70" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -10518,7 +10533,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="71" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -10537,7 +10552,7 @@
       <c r="BC71" s="48"/>
       <c r="BD71" s="48"/>
     </row>
-    <row r="72" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -10556,7 +10571,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="73" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -10579,7 +10594,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="74" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
@@ -10599,7 +10614,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="75" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
@@ -10622,7 +10637,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="76" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
@@ -10641,7 +10656,7 @@
       <c r="BC76" s="48"/>
       <c r="BD76" s="48"/>
     </row>
-    <row r="77" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
@@ -10657,7 +10672,7 @@
       <c r="BC77" s="47"/>
       <c r="BD77" s="47"/>
     </row>
-    <row r="78" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
@@ -10673,7 +10688,7 @@
       <c r="BC78" s="47"/>
       <c r="BD78" s="47"/>
     </row>
-    <row r="79" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
@@ -10689,7 +10704,7 @@
       <c r="BC79" s="47"/>
       <c r="BD79" s="47"/>
     </row>
-    <row r="80" spans="1:176" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:176" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
@@ -10709,7 +10724,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="81" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
@@ -10728,7 +10743,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="82" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
@@ -10744,7 +10759,7 @@
       <c r="BC82" s="42"/>
       <c r="BD82" s="42"/>
     </row>
-    <row r="83" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
@@ -10760,7 +10775,7 @@
       <c r="BC83" s="48"/>
       <c r="BD83" s="48"/>
     </row>
-    <row r="84" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
@@ -10776,7 +10791,7 @@
       <c r="BC84" s="40"/>
       <c r="BD84" s="41"/>
     </row>
-    <row r="85" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
@@ -10796,7 +10811,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="86" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
@@ -10816,7 +10831,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="87" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
@@ -10832,7 +10847,7 @@
       <c r="BC87" s="39"/>
       <c r="BD87" s="39"/>
     </row>
-    <row r="88" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
@@ -10887,7 +10902,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="89" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
@@ -10907,7 +10922,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="90" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
@@ -10950,7 +10965,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="91" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
@@ -10970,7 +10985,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="92" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
@@ -11026,7 +11041,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="93" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
@@ -11046,7 +11061,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="94" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
@@ -11066,7 +11081,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="95" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
@@ -11086,7 +11101,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="96" spans="1:199" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:199" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
@@ -11105,7 +11120,7 @@
       <c r="BC96" s="47"/>
       <c r="BD96" s="47"/>
     </row>
-    <row r="97" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
@@ -11146,7 +11161,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="98" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
@@ -11165,7 +11180,7 @@
       <c r="BC98" s="50"/>
       <c r="BD98" s="50"/>
     </row>
-    <row r="99" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>98</v>
       </c>
@@ -11181,7 +11196,7 @@
       <c r="BC99" s="47"/>
       <c r="BD99" s="47"/>
     </row>
-    <row r="100" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>99</v>
       </c>
@@ -11201,7 +11216,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="101" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>100</v>
       </c>
@@ -11221,7 +11236,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="102" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>101</v>
       </c>
@@ -11241,7 +11256,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="103" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>102</v>
       </c>
@@ -11257,7 +11272,7 @@
       <c r="BC103" s="47"/>
       <c r="BD103" s="47"/>
     </row>
-    <row r="104" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
         <v>103</v>
       </c>
@@ -11273,7 +11288,7 @@
       <c r="BC104" s="51"/>
       <c r="BD104" s="51"/>
     </row>
-    <row r="105" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>104</v>
       </c>
@@ -11289,7 +11304,7 @@
       <c r="BC105" s="52"/>
       <c r="BD105" s="52"/>
     </row>
-    <row r="106" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>105</v>
       </c>
@@ -11305,7 +11320,7 @@
       <c r="BC106" s="40"/>
       <c r="BD106" s="41"/>
     </row>
-    <row r="107" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -11325,7 +11340,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="108" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>107</v>
       </c>
@@ -11345,37 +11360,37 @@
         <v>676</v>
       </c>
     </row>
-    <row r="109" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
     </row>
-    <row r="110" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
     </row>
-    <row r="111" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
     </row>
-    <row r="112" spans="1:190" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:190" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -11439,157 +11454,157 @@
     <tabColor theme="9" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A2:V42"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" style="4" customWidth="1"/>
-    <col min="2" max="4" width="8.6328125" style="4"/>
-    <col min="5" max="5" width="12.36328125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="8.6328125" style="4"/>
-    <col min="7" max="7" width="8.6328125" style="4" customWidth="1"/>
-    <col min="8" max="16384" width="8.6328125" style="4"/>
+    <col min="1" max="1" width="10.33203125" style="4" customWidth="1"/>
+    <col min="2" max="4" width="8.6640625" style="4"/>
+    <col min="5" max="5" width="12.33203125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="4"/>
+    <col min="7" max="7" width="8.6640625" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="8.6640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:22" ht="21" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:22" ht="21" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>688</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>711</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>689</v>
       </c>
       <c r="R9" s="11"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>741</v>
       </c>
       <c r="V10" s="5"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>752</v>
       </c>
       <c r="S12" s="9"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="S13" s="9"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" s="18"/>
       <c r="S14" s="9"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="S15" s="9"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" s="10"/>
       <c r="S19" s="9"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="R20" s="5"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" s="10"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A22" s="11"/>
       <c r="R22" s="5"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23" s="11"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24" s="5"/>
       <c r="V24" s="15"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26" s="11"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="V27" s="5"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28" s="5"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" s="10"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" s="10"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31" s="10"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" s="10"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="10"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="10"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="16"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" s="5"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" s="14"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="5"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" s="10"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" s="17"/>
     </row>
   </sheetData>
@@ -11599,6 +11614,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x010100A603BB68AE5C0F4C908E70EB4D1DDDC3" ma:contentTypeVersion="15" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="bc1901b771652496ef02f4cbdf878f9e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95" xmlns:ns4="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6c61e44642a1e9e2aad865b2f0b39e8f" ns3:_="" ns4:_="">
     <xsd:import namespace="31ffec6e-e0c6-46d3-bf16-e7019fdf1f95"/>
@@ -11833,14 +11856,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11851,6 +11866,16 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27BF0A1B-B2BC-4159-BD4C-213AA0853490}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11869,16 +11894,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627ED23C-5EEB-4F10-AA20-79B788D8342E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="20b5f8f8-e964-4ea5-9bc5-5fa83731a92f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A16A6EDB-4C6A-433C-9B54-BF88B9AEEE87}">
   <ds:schemaRefs>

</xml_diff>